<commit_message>
Update Excel inventory workbook
</commit_message>
<xml_diff>
--- a/excel/SIOMS_Inventory.xlsx
+++ b/excel/SIOMS_Inventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\VI5PEPF000007D6\EXCELCNV\bf42e1fb-6199-4875-9a7e-67583808a727\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\VI5PEPF0000082D\EXCELCNV\0d7dcb2c-fded-4d1d-a8c4-c9bb1a0d778c\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{60AC8A63-81A7-4B35-A06F-4AAA462A2E80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{598CD421-3AA4-46CE-B674-A14531B56381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" xr2:uid="{3BDBB065-E3AF-489A-B7BE-4567A04EF8F9}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" xr2:uid="{82F17D93-7CAE-40E0-A3D6-5ED9C47C2871}"/>
   </bookViews>
   <sheets>
     <sheet name="in" sheetId="1" r:id="rId1"/>
@@ -604,6 +604,19 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1CE5CD73-5A90-496D-9E11-6802A85242DA}" name="Tablo1" displayName="Tablo1" ref="A1:D4" totalsRowShown="0">
+  <autoFilter ref="A1:D4" xr:uid="{1CE5CD73-5A90-496D-9E11-6802A85242DA}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{86D6A012-13F4-4F02-ACCE-BAD4DC02A81E}" name="name"/>
+    <tableColumn id="2" xr3:uid="{4927D3AF-E487-4AD3-BFFE-0D25D0B44A46}" name="category"/>
+    <tableColumn id="3" xr3:uid="{66E9D6F5-8159-4C1D-8713-8A5E3C25D4B0}" name="quantity"/>
+    <tableColumn id="4" xr3:uid="{44E07286-A76C-4030-B940-87C0CD96DB9C}" name="price"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -902,9 +915,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBAD44E2-DE46-4860-AC8E-A01941CEB561}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B94327E0-2804-433D-BC47-C09DB4F9F29E}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
@@ -964,5 +982,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>